<commit_message>
Deploying to gh-pages from @ mattaq31/Hash-CAD@5fe914dfae4f6a24bbef6159c082ae6b7644111f 🚀
</commit_message>
<xml_diff>
--- a/plates/cargo_plates/P3510_SSW_cnt_patterning.xlsx
+++ b/plates/cargo_plates/P3510_SSW_cnt_patterning.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10322"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/matt/Documents/Shih_Lab_Postdoc/research_projects/crisscross_code/crisscross_kit/crisscross/dna_source_plates/cargo_plates/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stellawang/Documents/gitrepos/Crisscross-Design/crisscross_kit/crisscross/dna_source_plates/cargo_plates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3211A15B-4D38-6244-9687-48E82E1F3E09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B05911FD-561F-154F-B8CE-FA8DEA67AF1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="620" windowWidth="51200" windowHeight="28180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-10540" yWindow="-25700" windowWidth="47420" windowHeight="21300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="All Data" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1015" uniqueCount="753">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1026" uniqueCount="757">
   <si>
     <t>well</t>
   </si>
@@ -2274,20 +2274,32 @@
     <t>P</t>
   </si>
   <si>
-    <t>Cargo Handle For Slat Position 20, Side h2, Cargo ID SW066GoldNanowireAntiHandle10nt</t>
-  </si>
-  <si>
-    <t>CARGO-SW066GoldNanowireAntiHandle10nt-h2-position_20</t>
-  </si>
-  <si>
-    <t>TATAGCCCGGAACCTCATTTTCAGGGATAGCCTCATAGTTAG tt ATAAAAGCAT</t>
+    <t>CATTTTTGCGGAATTCCATATAACAGTTGAATTTGGGGCGCG tt ATAAAAGCAT</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 12, Side h2, Cargo ID SW066GoldNanowireAntiHandle10nt, ordered as SSW109</t>
+  </si>
+  <si>
+    <t>CARGO-SW066GoldNanowireAntiHandle10nt-h2-position_12</t>
+  </si>
+  <si>
+    <t>NON-SLAT OLIGO</t>
+  </si>
+  <si>
+    <t>TTTTTTTTTT</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>Obsolete well, may be contaminated, do not use</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2303,8 +2315,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2320,6 +2338,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF0000FF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD3D3D3"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2351,13 +2375,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4619,13 +4646,13 @@
         <v>222</v>
       </c>
       <c r="B219" t="s">
-        <v>459</v>
+        <v>753</v>
       </c>
       <c r="C219" t="s">
         <v>565</v>
       </c>
       <c r="D219" t="s">
-        <v>673</v>
+        <v>756</v>
       </c>
       <c r="E219">
         <v>200</v>
@@ -4653,13 +4680,13 @@
         <v>224</v>
       </c>
       <c r="B221" t="s">
-        <v>751</v>
+        <v>753</v>
       </c>
       <c r="C221" t="s">
-        <v>752</v>
+        <v>754</v>
       </c>
       <c r="D221" t="s">
-        <v>750</v>
+        <v>756</v>
       </c>
       <c r="E221">
         <v>200</v>
@@ -4674,10 +4701,34 @@
       <c r="A223" t="s">
         <v>226</v>
       </c>
+      <c r="B223" t="s">
+        <v>459</v>
+      </c>
+      <c r="C223" t="s">
+        <v>565</v>
+      </c>
+      <c r="D223" t="s">
+        <v>673</v>
+      </c>
+      <c r="E223">
+        <v>200</v>
+      </c>
     </row>
     <row r="224" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A224" t="s">
         <v>227</v>
+      </c>
+      <c r="B224" t="s">
+        <v>752</v>
+      </c>
+      <c r="C224" s="4" t="s">
+        <v>750</v>
+      </c>
+      <c r="D224" t="s">
+        <v>751</v>
+      </c>
+      <c r="E224">
+        <v>200</v>
       </c>
     </row>
     <row r="225" spans="1:1" x14ac:dyDescent="0.2">
@@ -5930,8 +5981,7 @@
     <col min="1" max="1" width="53.6640625" customWidth="1"/>
     <col min="2" max="3" width="54.6640625" customWidth="1"/>
     <col min="4" max="4" width="45.6640625" customWidth="1"/>
-    <col min="5" max="5" width="52.33203125" customWidth="1"/>
-    <col min="6" max="6" width="41.6640625" customWidth="1"/>
+    <col min="5" max="6" width="41.6640625" customWidth="1"/>
     <col min="7" max="8" width="45.6640625" customWidth="1"/>
     <col min="9" max="9" width="41.6640625" customWidth="1"/>
     <col min="10" max="10" width="37.6640625" customWidth="1"/>
@@ -6281,13 +6331,19 @@
         <v>458</v>
       </c>
       <c r="C11" t="s">
-        <v>459</v>
+        <v>753</v>
       </c>
       <c r="D11" t="s">
         <v>460</v>
       </c>
       <c r="E11" t="s">
-        <v>751</v>
+        <v>753</v>
+      </c>
+      <c r="G11" t="s">
+        <v>459</v>
+      </c>
+      <c r="H11" t="s">
+        <v>752</v>
       </c>
     </row>
     <row r="12" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.2">
@@ -6777,10 +6833,19 @@
       <c r="B11" s="3" t="s">
         <v>736</v>
       </c>
-      <c r="C11" s="3" t="s">
-        <v>736</v>
+      <c r="C11" s="6" t="s">
+        <v>755</v>
       </c>
       <c r="D11" s="3" t="s">
+        <v>736</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>755</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>736</v>
+      </c>
+      <c r="H11" s="5" t="s">
         <v>736</v>
       </c>
     </row>

</xml_diff>